<commit_message>
Working Commit - cfr-eng -> scimago ( 257 data - 6 minutes )
</commit_message>
<xml_diff>
--- a/output/scimago_results.xlsx
+++ b/output/scimago_results.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>1.56</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="3">
@@ -542,7 +542,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>1.37</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="4">
@@ -583,7 +583,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>1.65</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="5">
@@ -624,7 +624,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>1.66</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="6">
@@ -665,7 +665,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>1.17</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="7">
@@ -706,7 +706,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>1.36</v>
+        <v>2.28</v>
       </c>
     </row>
     <row r="8">
@@ -747,7 +747,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>1.36</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="9">
@@ -788,7 +788,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>1.58</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="10">
@@ -829,7 +829,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>1.2</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="11">
@@ -870,7 +870,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>1.2</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -911,7 +911,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>1.19</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="13">
@@ -952,7 +952,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>1.12</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="14">
@@ -993,7 +993,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>1.38</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="15">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>1.16</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="16">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>0.85</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="17">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>1.18</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="18">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>1.31</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="19">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
-        <v>1.49</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="20">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>1.47</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="21">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
-        <v>1.19</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="22">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
-        <v>1.09</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="23">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="n">
-        <v>1.51</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="24">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="n">
-        <v>1.39</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="25">
@@ -1448,7 +1448,7 @@
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
-        <v>1.38</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="26">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
-        <v>1.76</v>
+        <v>2.06</v>
       </c>
     </row>
     <row r="27">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="n">
-        <v>1.39</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="28">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="n">
-        <v>1.47</v>
+        <v>1.26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>